<commit_message>
updated to DAC/ADC & pre-amp on BOM
</commit_message>
<xml_diff>
--- a/fpga_guitar_pedal_bom.xlsx
+++ b/fpga_guitar_pedal_bom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\Summer 26 FPGA Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80E740ED-B699-48BE-9056-ED895C301AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBAF9795-3347-489F-9C64-C2D27FB578C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="113">
   <si>
     <t>Category</t>
   </si>
@@ -214,15 +214,6 @@
     <t>Zynq-7000 SoC dev board (XC7Z020), 512MB DDR3, extra FPGA resources</t>
   </si>
   <si>
-    <t>Larger Zynq-7020 device gives more headroom for parallel FX blocks and higher oversampling while keeping same board footprint.</t>
-  </si>
-  <si>
-    <t>Same ADC as budget build keeps firmware/HDL identical; still good enough for many guitar FX.</t>
-  </si>
-  <si>
-    <t>Keeps high-resolution output path; you can experiment with dither/oversampling on the larger FPGA.</t>
-  </si>
-  <si>
     <t>Primary UI control for navigating presets and tweaking parameters.</t>
   </si>
   <si>
@@ -359,16 +350,48 @@
   </si>
   <si>
     <t>Knobs, dress nuts, standoffs, cable glands (estimated)</t>
+  </si>
+  <si>
+    <t>Digilent Pmod I2S2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2-ch 24-bit I2S ADC module for audio input, 108kHz </t>
+  </si>
+  <si>
+    <t>https://www.digikey.ca/en/products/detail/digilent-inc/410-346-20/6674366</t>
+  </si>
+  <si>
+    <t>LINK</t>
+  </si>
+  <si>
+    <t>410-379 Digilent, Inc. | Expansion Boards, Daughter Cards | DigiKey</t>
+  </si>
+  <si>
+    <t>z-10 is only like $360</t>
+  </si>
+  <si>
+    <t>Pre-Amp</t>
+  </si>
+  <si>
+    <t>Lower impedance &amp; boost weak signal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -391,10 +414,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="45"/>
@@ -402,8 +426,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="45"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -436,9 +462,9 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="ValueBOM" displayName="ValueBOM" ref="B1:H20">
-  <autoFilter ref="B1:H20" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="ValueBOM" displayName="ValueBOM" ref="B1:I21">
+  <autoFilter ref="B1:I21" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Category"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Item"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Description"/>
@@ -446,6 +472,7 @@
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Unit Price (CAD)"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Ext Cost (CAD)"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Notes / Reason"/>
+    <tableColumn id="8" xr3:uid="{C9F51080-3B89-4D3D-8A93-01F914543D18}" name="LINK"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1125,7 +1152,7 @@
     </row>
     <row r="17" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E17" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F17">
         <f>SUM(BudgetBOM[Ext Cost (CAD)])</f>
@@ -1142,7 +1169,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -1152,9 +1179,10 @@
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="117.42578125" customWidth="1"/>
+    <col min="9" max="9" width="69.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -1176,10 +1204,13 @@
       <c r="H1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
@@ -1194,40 +1225,45 @@
         <v>1</v>
       </c>
       <c r="F2">
-        <v>397.6</v>
+        <v>501.07</v>
       </c>
       <c r="G2">
-        <v>397.6</v>
+        <f>ValueBOM[[#This Row],[Unit Price (CAD)]]*ValueBOM[[#This Row],[Qty]]</f>
+        <v>501.07</v>
       </c>
       <c r="H2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" t="s">
         <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>105</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F3">
-        <v>39.76</v>
+        <v>43.29</v>
       </c>
       <c r="G3">
-        <v>39.76</v>
-      </c>
-      <c r="H3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <f>ValueBOM[[#This Row],[Unit Price (CAD)]]*ValueBOM[[#This Row],[Qty]]</f>
+        <v>21.645</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" t="s">
         <v>11</v>
@@ -1239,31 +1275,32 @@
         <v>16</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F4">
-        <v>39.76</v>
+        <v>43.29</v>
       </c>
       <c r="G4">
-        <v>39.76</v>
-      </c>
-      <c r="H4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <f>ValueBOM[[#This Row],[Unit Price (CAD)]]*ValueBOM[[#This Row],[Qty]]</f>
+        <v>21.645</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B6" t="s">
         <v>18</v>
       </c>
       <c r="G6">
-        <f t="shared" ref="G6:G20" si="0">E6*F6</f>
+        <f t="shared" ref="G6:G21" si="0">E6*F6</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" t="s">
         <v>18</v>
@@ -1285,10 +1322,10 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" t="s">
         <v>18</v>
@@ -1310,15 +1347,15 @@
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B10" t="s">
         <v>28</v>
@@ -1340,19 +1377,19 @@
         <v>6</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" t="s">
         <v>28</v>
       </c>
       <c r="C11" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D11" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -1365,15 +1402,15 @@
         <v>3.3</v>
       </c>
       <c r="H11" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B13" t="s">
         <v>32</v>
@@ -1395,118 +1432,130 @@
         <v>25</v>
       </c>
       <c r="H13" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" t="s">
         <v>32</v>
       </c>
       <c r="C14" t="s">
+        <v>111</v>
+      </c>
+      <c r="D14" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" t="s">
         <v>36</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D15" t="s">
         <v>37</v>
       </c>
-      <c r="E14">
+      <c r="E15">
         <v>0</v>
       </c>
-      <c r="F14">
+      <c r="F15">
         <v>3</v>
       </c>
-      <c r="G14">
-        <f>E14*F14</f>
+      <c r="G15">
+        <f>E15*F15</f>
         <v>0</v>
       </c>
-      <c r="H14" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
+      <c r="H15" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
         <v>39</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C17" t="s">
         <v>43</v>
       </c>
-      <c r="D16" t="s">
-        <v>107</v>
-      </c>
-      <c r="E16">
-        <v>1</v>
-      </c>
-      <c r="F16">
+      <c r="D17" t="s">
+        <v>104</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
         <v>30</v>
       </c>
-      <c r="G16">
+      <c r="G17">
         <v>30</v>
       </c>
-      <c r="H16" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B18" t="s">
+      <c r="H17" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" t="s">
         <v>46</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C19" t="s">
         <v>47</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D19" t="s">
         <v>48</v>
       </c>
-      <c r="E18">
-        <v>1</v>
-      </c>
-      <c r="F18">
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
         <v>0</v>
       </c>
-      <c r="G18">
+      <c r="G19">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
+      <c r="H19" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
         <v>50</v>
       </c>
-      <c r="C20" t="s">
-        <v>106</v>
-      </c>
-      <c r="E20">
-        <v>1</v>
-      </c>
-      <c r="F20">
+      <c r="C21" t="s">
+        <v>103</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
         <v>30</v>
       </c>
-      <c r="G20">
+      <c r="G21">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="F22" t="s">
-        <v>101</v>
-      </c>
-      <c r="G22">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F23" t="s">
+        <v>98</v>
+      </c>
+      <c r="G23">
         <f>SUM(ValueBOM[Ext Cost (CAD)])</f>
-        <v>571.42000000000007</v>
-      </c>
-    </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="F24" t="s">
-        <v>102</v>
-      </c>
-      <c r="G24">
+        <v>638.66</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="F25" t="s">
+        <v>99</v>
+      </c>
+      <c r="G25">
         <f>SUM(G2:G4)</f>
-        <v>477.12</v>
+        <v>544.36</v>
       </c>
     </row>
   </sheetData>
@@ -1514,11 +1563,16 @@
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="A10:A11"/>
-    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="A13:A15"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1" xr:uid="{6324B0F3-E717-4E98-A730-1E2B32763DC4}"/>
+    <hyperlink ref="I4" r:id="rId2" display="https://www.digikey.ca/en/products/detail/digilent-inc/410-379/9445907" xr:uid="{F24DC25F-D6AD-49B0-8CC6-2B98E6F7A37A}"/>
+    <hyperlink ref="I3" r:id="rId3" display="https://www.digikey.ca/en/products/detail/digilent-inc/410-379/9445907" xr:uid="{9A8A63BE-CDC0-43E6-A2E6-BE2A75A73942}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1581,7 +1635,7 @@
         <v>436.46</v>
       </c>
       <c r="G2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1605,7 +1659,7 @@
         <v>43.19</v>
       </c>
       <c r="G3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1629,7 +1683,7 @@
         <v>41.09</v>
       </c>
       <c r="G4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1653,7 +1707,7 @@
         <v>5.25</v>
       </c>
       <c r="G5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1664,7 +1718,7 @@
         <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1677,7 +1731,7 @@
         <v>6</v>
       </c>
       <c r="G6" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1685,10 +1739,10 @@
         <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D7">
         <v>2</v>
@@ -1701,7 +1755,7 @@
         <v>12.02</v>
       </c>
       <c r="G7" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1709,10 +1763,10 @@
         <v>28</v>
       </c>
       <c r="B8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C8" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1725,7 +1779,7 @@
         <v>13.28</v>
       </c>
       <c r="G8" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1733,10 +1787,10 @@
         <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C9" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -1749,7 +1803,7 @@
         <v>3.3</v>
       </c>
       <c r="G9" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -1760,7 +1814,7 @@
         <v>33</v>
       </c>
       <c r="C10" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1773,7 +1827,7 @@
         <v>35</v>
       </c>
       <c r="G10" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1797,7 +1851,7 @@
         <v>2.99</v>
       </c>
       <c r="G11" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1805,10 +1859,10 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1821,7 +1875,7 @@
         <v>18.989999999999998</v>
       </c>
       <c r="G12" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1829,10 +1883,10 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C13" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1845,7 +1899,7 @@
         <v>60</v>
       </c>
       <c r="G13" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1869,7 +1923,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1877,10 +1931,10 @@
         <v>50</v>
       </c>
       <c r="B15" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C15" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1893,7 +1947,7 @@
         <v>189.9</v>
       </c>
       <c r="G15" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1917,12 +1971,12 @@
         <v>25.87</v>
       </c>
       <c r="G16" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E18" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F18">
         <f>SUM(HighQualityBOM[Ext Cost (CAD)])</f>

</xml_diff>